<commit_message>
Deploying to gh-pages from @ eurovibes/pors485@1cf3faf7323da217d3328c908e8c2efa7589ea1e 🚀
</commit_message>
<xml_diff>
--- a/Fabrication/BoM/pors485-bom_0.1.xlsx
+++ b/Fabrication/BoM/pors485-bom_0.1.xlsx
@@ -370,10 +370,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>647710</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>95260</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>3526378</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>173578</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -400,7 +400,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="4876810" cy="4876810"/>
+          <a:ext cx="15242128" cy="15242128"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>